<commit_message>
Update SkyportCare roadmap workbook; add Digital Platforms Business Model xlsx
Made-with: Cursor
</commit_message>
<xml_diff>
--- a/SkyportCare_Roadmap.xlsx
+++ b/SkyportCare_Roadmap.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/vishwas/Documents/DevelopmentProjects/Skyport-Web/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{E22810F2-23E3-3E4C-B92C-DEDEF57B99D6}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{02EB0C24-E4DE-DE40-8B67-0A7E7E6BD8AA}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="56000" yWindow="840" windowWidth="42440" windowHeight="25380" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="0" yWindow="760" windowWidth="30240" windowHeight="17760" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Summary" sheetId="2" r:id="rId1"/>
@@ -38,7 +38,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="289" uniqueCount="88">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="301" uniqueCount="90">
   <si>
     <t>Feature Group</t>
   </si>
@@ -425,6 +425,12 @@
   </si>
   <si>
     <t>Ability for dealers to submit feature requests intuitively</t>
+  </si>
+  <si>
+    <t>ROI &amp; $ Savings Insights (avoided service calls, failure prevention, optimization impact)</t>
+  </si>
+  <si>
+    <t>Actionable Alerts (root cause, impact, recommended action)</t>
   </si>
 </sst>
 </file>
@@ -928,10 +934,10 @@
                 <c:formatCode>0%</c:formatCode>
                 <c:ptCount val="3"/>
                 <c:pt idx="1">
-                  <c:v>0.69444444444444442</c:v>
+                  <c:v>0.72222222222222221</c:v>
                 </c:pt>
                 <c:pt idx="2">
-                  <c:v>0.30555555555555558</c:v>
+                  <c:v>0.33333333333333331</c:v>
                 </c:pt>
               </c:numCache>
             </c:numRef>
@@ -1205,10 +1211,10 @@
                   <c:v>0.19444444444444445</c:v>
                 </c:pt>
                 <c:pt idx="2">
-                  <c:v>0.30555555555555558</c:v>
+                  <c:v>0.33333333333333331</c:v>
                 </c:pt>
                 <c:pt idx="3">
-                  <c:v>0.22222222222222221</c:v>
+                  <c:v>0.25</c:v>
                 </c:pt>
                 <c:pt idx="4">
                   <c:v>0.16666666666666666</c:v>
@@ -1496,10 +1502,10 @@
                   <c:v>0</c:v>
                 </c:pt>
                 <c:pt idx="3">
-                  <c:v>0.63888888888888884</c:v>
+                  <c:v>0.66666666666666663</c:v>
                 </c:pt>
                 <c:pt idx="4">
-                  <c:v>0.22222222222222221</c:v>
+                  <c:v>0.25</c:v>
                 </c:pt>
                 <c:pt idx="5">
                   <c:v>5.5555555555555552E-2</c:v>
@@ -3727,8 +3733,8 @@
         <v>7</v>
       </c>
       <c r="B2" s="20">
-        <f>SkyportCare!D54</f>
-        <v>0.69444444444444442</v>
+        <f>SkyportCare!D56</f>
+        <v>0.72222222222222221</v>
       </c>
     </row>
     <row r="3" spans="1:2" x14ac:dyDescent="0.2">
@@ -3736,8 +3742,8 @@
         <v>22</v>
       </c>
       <c r="B3" s="20">
-        <f>SkyportCare!D55</f>
-        <v>0.30555555555555558</v>
+        <f>SkyportCare!D57</f>
+        <v>0.33333333333333331</v>
       </c>
     </row>
     <row r="4" spans="1:2" ht="16" customHeight="1" x14ac:dyDescent="0.2">
@@ -3751,7 +3757,7 @@
         <v>19</v>
       </c>
       <c r="B5" s="22">
-        <f>SkyportCare!D47</f>
+        <f>SkyportCare!D49</f>
         <v>0.1111111111111111</v>
       </c>
     </row>
@@ -3760,7 +3766,7 @@
         <v>20</v>
       </c>
       <c r="B6" s="22">
-        <f>SkyportCare!D48</f>
+        <f>SkyportCare!D50</f>
         <v>0.19444444444444445</v>
       </c>
     </row>
@@ -3769,8 +3775,8 @@
         <v>6</v>
       </c>
       <c r="B7" s="22">
-        <f>SkyportCare!D49</f>
-        <v>0.30555555555555558</v>
+        <f>SkyportCare!D51</f>
+        <v>0.33333333333333331</v>
       </c>
     </row>
     <row r="8" spans="1:2" x14ac:dyDescent="0.2">
@@ -3778,8 +3784,8 @@
         <v>17</v>
       </c>
       <c r="B8" s="22">
-        <f>SkyportCare!D50</f>
-        <v>0.22222222222222221</v>
+        <f>SkyportCare!D52</f>
+        <v>0.25</v>
       </c>
     </row>
     <row r="9" spans="1:2" x14ac:dyDescent="0.2">
@@ -3787,7 +3793,7 @@
         <v>21</v>
       </c>
       <c r="B9" s="22">
-        <f>SkyportCare!D51</f>
+        <f>SkyportCare!D53</f>
         <v>0.16666666666666666</v>
       </c>
     </row>
@@ -3806,7 +3812,7 @@
         <v>8</v>
       </c>
       <c r="B12" s="22">
-        <f>SkyportCare!E39</f>
+        <f>SkyportCare!E41</f>
         <v>2.7777777777777776E-2</v>
       </c>
     </row>
@@ -3815,7 +3821,7 @@
         <v>10</v>
       </c>
       <c r="B13" s="22">
-        <f>SkyportCare!E40</f>
+        <f>SkyportCare!E42</f>
         <v>5.5555555555555552E-2</v>
       </c>
     </row>
@@ -3824,7 +3830,7 @@
         <v>11</v>
       </c>
       <c r="B14" s="22">
-        <f>SkyportCare!E41</f>
+        <f>SkyportCare!E43</f>
         <v>0</v>
       </c>
     </row>
@@ -3833,8 +3839,8 @@
         <v>13</v>
       </c>
       <c r="B15" s="22">
-        <f>SkyportCare!E42</f>
-        <v>0.63888888888888884</v>
+        <f>SkyportCare!E44</f>
+        <v>0.66666666666666663</v>
       </c>
     </row>
     <row r="16" spans="1:2" ht="16" x14ac:dyDescent="0.2">
@@ -3842,8 +3848,8 @@
         <v>15</v>
       </c>
       <c r="B16" s="22">
-        <f>SkyportCare!E43</f>
-        <v>0.22222222222222221</v>
+        <f>SkyportCare!E45</f>
+        <v>0.25</v>
       </c>
     </row>
     <row r="17" spans="1:2" ht="16" x14ac:dyDescent="0.2">
@@ -3851,7 +3857,7 @@
         <v>16</v>
       </c>
       <c r="B17" s="22">
-        <f>SkyportCare!E44</f>
+        <f>SkyportCare!E46</f>
         <v>5.5555555555555552E-2</v>
       </c>
     </row>
@@ -3868,7 +3874,7 @@
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{94DC2D9C-A4B6-774F-B8A7-9331E3148EF8}">
-  <dimension ref="A1:H55"/>
+  <dimension ref="A1:H57"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="8.83203125" defaultRowHeight="15" x14ac:dyDescent="0.2"/>
   <cols>
     <col min="1" max="1" width="21.1640625" style="1" customWidth="1"/>
@@ -4174,60 +4180,60 @@
         <v>76</v>
       </c>
     </row>
-    <row r="13" spans="1:8" ht="16" x14ac:dyDescent="0.2">
+    <row r="13" spans="1:8" ht="20" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A13" s="39"/>
       <c r="B13" s="6" t="s">
+        <v>89</v>
+      </c>
+      <c r="C13" s="7" t="s">
+        <v>13</v>
+      </c>
+      <c r="D13" s="7" t="s">
+        <v>6</v>
+      </c>
+      <c r="E13" s="10" t="s">
+        <v>7</v>
+      </c>
+      <c r="F13" s="28" t="s">
+        <v>84</v>
+      </c>
+      <c r="G13" s="5">
+        <v>2</v>
+      </c>
+      <c r="H13" s="5" t="s">
+        <v>75</v>
+      </c>
+    </row>
+    <row r="14" spans="1:8" ht="16" x14ac:dyDescent="0.2">
+      <c r="A14" s="39"/>
+      <c r="B14" s="6" t="s">
         <v>58</v>
       </c>
-      <c r="C13" s="7" t="s">
+      <c r="C14" s="7" t="s">
         <v>15</v>
       </c>
-      <c r="D13" s="7" t="s">
+      <c r="D14" s="7" t="s">
         <v>17</v>
       </c>
-      <c r="E13" s="28" t="s">
+      <c r="E14" s="28" t="s">
         <v>22</v>
       </c>
-      <c r="F13" s="28" t="s">
+      <c r="F14" s="28" t="s">
         <v>83</v>
       </c>
-      <c r="G13" s="5">
+      <c r="G14" s="5">
         <v>3</v>
       </c>
-      <c r="H13" s="5" t="s">
+      <c r="H14" s="5" t="s">
         <v>76</v>
       </c>
     </row>
-    <row r="14" spans="1:8" ht="15" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A14" s="35" t="s">
+    <row r="15" spans="1:8" ht="15" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A15" s="35" t="s">
         <v>40</v>
       </c>
-      <c r="B14" s="23" t="s">
+      <c r="B15" s="23" t="s">
         <v>27</v>
-      </c>
-      <c r="C14" s="7" t="s">
-        <v>13</v>
-      </c>
-      <c r="D14" s="7" t="s">
-        <v>6</v>
-      </c>
-      <c r="E14" s="10" t="s">
-        <v>7</v>
-      </c>
-      <c r="F14" s="28" t="s">
-        <v>82</v>
-      </c>
-      <c r="G14" s="5">
-        <v>1</v>
-      </c>
-      <c r="H14" s="5" t="s">
-        <v>75</v>
-      </c>
-    </row>
-    <row r="15" spans="1:8" ht="15" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A15" s="36"/>
-      <c r="B15" s="6" t="s">
-        <v>67</v>
       </c>
       <c r="C15" s="7" t="s">
         <v>13</v>
@@ -4239,10 +4245,10 @@
         <v>7</v>
       </c>
       <c r="F15" s="28" t="s">
-        <v>84</v>
+        <v>82</v>
       </c>
       <c r="G15" s="5">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="H15" s="5" t="s">
         <v>75</v>
@@ -4251,19 +4257,19 @@
     <row r="16" spans="1:8" ht="15" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A16" s="36"/>
       <c r="B16" s="6" t="s">
-        <v>49</v>
+        <v>67</v>
       </c>
       <c r="C16" s="7" t="s">
-        <v>10</v>
+        <v>13</v>
       </c>
       <c r="D16" s="7" t="s">
-        <v>19</v>
+        <v>6</v>
       </c>
       <c r="E16" s="10" t="s">
         <v>7</v>
       </c>
       <c r="F16" s="28" t="s">
-        <v>83</v>
+        <v>84</v>
       </c>
       <c r="G16" s="5">
         <v>2</v>
@@ -4273,15 +4279,15 @@
       </c>
     </row>
     <row r="17" spans="1:8" ht="15" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A17" s="37"/>
+      <c r="A17" s="36"/>
       <c r="B17" s="6" t="s">
-        <v>50</v>
+        <v>49</v>
       </c>
       <c r="C17" s="7" t="s">
-        <v>13</v>
+        <v>10</v>
       </c>
       <c r="D17" s="7" t="s">
-        <v>6</v>
+        <v>19</v>
       </c>
       <c r="E17" s="10" t="s">
         <v>7</v>
@@ -4296,24 +4302,22 @@
         <v>75</v>
       </c>
     </row>
-    <row r="18" spans="1:8" ht="31" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A18" s="39" t="s">
-        <v>34</v>
-      </c>
+    <row r="18" spans="1:8" ht="15" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A18" s="37"/>
       <c r="B18" s="6" t="s">
-        <v>38</v>
+        <v>50</v>
       </c>
       <c r="C18" s="7" t="s">
         <v>13</v>
       </c>
       <c r="D18" s="7" t="s">
-        <v>19</v>
+        <v>6</v>
       </c>
       <c r="E18" s="10" t="s">
         <v>7</v>
       </c>
       <c r="F18" s="28" t="s">
-        <v>84</v>
+        <v>83</v>
       </c>
       <c r="G18" s="5">
         <v>2</v>
@@ -4322,10 +4326,12 @@
         <v>75</v>
       </c>
     </row>
-    <row r="19" spans="1:8" ht="19" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A19" s="39"/>
+    <row r="19" spans="1:8" ht="31" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A19" s="39" t="s">
+        <v>34</v>
+      </c>
       <c r="B19" s="6" t="s">
-        <v>35</v>
+        <v>38</v>
       </c>
       <c r="C19" s="7" t="s">
         <v>13</v>
@@ -4346,19 +4352,19 @@
         <v>75</v>
       </c>
     </row>
-    <row r="20" spans="1:8" ht="16" x14ac:dyDescent="0.2">
+    <row r="20" spans="1:8" ht="19" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A20" s="39"/>
       <c r="B20" s="6" t="s">
-        <v>36</v>
+        <v>35</v>
       </c>
       <c r="C20" s="7" t="s">
-        <v>15</v>
+        <v>13</v>
       </c>
       <c r="D20" s="7" t="s">
         <v>19</v>
       </c>
       <c r="E20" s="10" t="s">
-        <v>22</v>
+        <v>7</v>
       </c>
       <c r="F20" s="28" t="s">
         <v>84</v>
@@ -4370,48 +4376,46 @@
         <v>75</v>
       </c>
     </row>
-    <row r="21" spans="1:8" ht="16" x14ac:dyDescent="0.2">
+    <row r="21" spans="1:8" ht="19" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A21" s="39"/>
-      <c r="B21" s="23" t="s">
-        <v>39</v>
+      <c r="B21" s="6" t="s">
+        <v>88</v>
       </c>
       <c r="C21" s="7" t="s">
-        <v>13</v>
+        <v>15</v>
       </c>
       <c r="D21" s="7" t="s">
         <v>17</v>
       </c>
-      <c r="E21" s="10" t="s">
-        <v>7</v>
+      <c r="E21" s="28" t="s">
+        <v>22</v>
       </c>
       <c r="F21" s="28" t="s">
-        <v>81</v>
+        <v>83</v>
       </c>
       <c r="G21" s="5">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="H21" s="5" t="s">
-        <v>75</v>
+        <v>76</v>
       </c>
     </row>
     <row r="22" spans="1:8" ht="16" x14ac:dyDescent="0.2">
-      <c r="A22" s="35" t="s">
-        <v>41</v>
-      </c>
+      <c r="A22" s="39"/>
       <c r="B22" s="6" t="s">
-        <v>68</v>
-      </c>
-      <c r="C22" s="4" t="s">
-        <v>8</v>
+        <v>36</v>
+      </c>
+      <c r="C22" s="7" t="s">
+        <v>15</v>
       </c>
       <c r="D22" s="7" t="s">
-        <v>20</v>
+        <v>19</v>
       </c>
       <c r="E22" s="10" t="s">
-        <v>7</v>
+        <v>22</v>
       </c>
       <c r="F22" s="28" t="s">
-        <v>85</v>
+        <v>84</v>
       </c>
       <c r="G22" s="5">
         <v>2</v>
@@ -4420,46 +4424,48 @@
         <v>75</v>
       </c>
     </row>
-    <row r="23" spans="1:8" ht="99" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A23" s="36"/>
-      <c r="B23" s="6" t="s">
-        <v>44</v>
+    <row r="23" spans="1:8" ht="16" x14ac:dyDescent="0.2">
+      <c r="A23" s="39"/>
+      <c r="B23" s="23" t="s">
+        <v>39</v>
       </c>
       <c r="C23" s="7" t="s">
         <v>13</v>
       </c>
       <c r="D23" s="7" t="s">
-        <v>6</v>
+        <v>17</v>
       </c>
       <c r="E23" s="10" t="s">
         <v>7</v>
       </c>
       <c r="F23" s="28" t="s">
-        <v>84</v>
+        <v>81</v>
       </c>
       <c r="G23" s="5">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="H23" s="5" t="s">
         <v>75</v>
       </c>
     </row>
-    <row r="24" spans="1:8" ht="186" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A24" s="36"/>
+    <row r="24" spans="1:8" ht="16" x14ac:dyDescent="0.2">
+      <c r="A24" s="35" t="s">
+        <v>41</v>
+      </c>
       <c r="B24" s="6" t="s">
-        <v>43</v>
-      </c>
-      <c r="C24" s="7" t="s">
-        <v>13</v>
+        <v>68</v>
+      </c>
+      <c r="C24" s="4" t="s">
+        <v>8</v>
       </c>
       <c r="D24" s="7" t="s">
-        <v>17</v>
+        <v>20</v>
       </c>
       <c r="E24" s="10" t="s">
         <v>7</v>
       </c>
       <c r="F24" s="28" t="s">
-        <v>84</v>
+        <v>85</v>
       </c>
       <c r="G24" s="5">
         <v>2</v>
@@ -4468,16 +4474,16 @@
         <v>75</v>
       </c>
     </row>
-    <row r="25" spans="1:8" ht="409" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A25" s="37"/>
+    <row r="25" spans="1:8" ht="99" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A25" s="36"/>
       <c r="B25" s="6" t="s">
-        <v>51</v>
+        <v>44</v>
       </c>
       <c r="C25" s="7" t="s">
         <v>13</v>
       </c>
       <c r="D25" s="7" t="s">
-        <v>17</v>
+        <v>6</v>
       </c>
       <c r="E25" s="10" t="s">
         <v>7</v>
@@ -4492,24 +4498,22 @@
         <v>75</v>
       </c>
     </row>
-    <row r="26" spans="1:8" ht="16" x14ac:dyDescent="0.2">
-      <c r="A26" s="39" t="s">
-        <v>42</v>
-      </c>
+    <row r="26" spans="1:8" ht="186" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A26" s="36"/>
       <c r="B26" s="6" t="s">
-        <v>55</v>
+        <v>43</v>
       </c>
       <c r="C26" s="7" t="s">
         <v>13</v>
       </c>
       <c r="D26" s="7" t="s">
-        <v>20</v>
+        <v>17</v>
       </c>
       <c r="E26" s="10" t="s">
         <v>7</v>
       </c>
       <c r="F26" s="28" t="s">
-        <v>85</v>
+        <v>84</v>
       </c>
       <c r="G26" s="5">
         <v>2</v>
@@ -4518,22 +4522,22 @@
         <v>75</v>
       </c>
     </row>
-    <row r="27" spans="1:8" ht="16" x14ac:dyDescent="0.2">
-      <c r="A27" s="39"/>
+    <row r="27" spans="1:8" ht="409" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A27" s="37"/>
       <c r="B27" s="6" t="s">
-        <v>52</v>
+        <v>51</v>
       </c>
       <c r="C27" s="7" t="s">
-        <v>15</v>
+        <v>13</v>
       </c>
       <c r="D27" s="7" t="s">
-        <v>6</v>
+        <v>17</v>
       </c>
       <c r="E27" s="10" t="s">
         <v>7</v>
       </c>
       <c r="F27" s="28" t="s">
-        <v>85</v>
+        <v>84</v>
       </c>
       <c r="G27" s="5">
         <v>2</v>
@@ -4543,18 +4547,20 @@
       </c>
     </row>
     <row r="28" spans="1:8" ht="16" x14ac:dyDescent="0.2">
-      <c r="A28" s="39"/>
+      <c r="A28" s="39" t="s">
+        <v>42</v>
+      </c>
       <c r="B28" s="6" t="s">
-        <v>53</v>
+        <v>55</v>
       </c>
       <c r="C28" s="7" t="s">
-        <v>15</v>
+        <v>13</v>
       </c>
       <c r="D28" s="7" t="s">
         <v>20</v>
       </c>
-      <c r="E28" s="28" t="s">
-        <v>22</v>
+      <c r="E28" s="10" t="s">
+        <v>7</v>
       </c>
       <c r="F28" s="28" t="s">
         <v>85</v>
@@ -4569,13 +4575,13 @@
     <row r="29" spans="1:8" ht="16" x14ac:dyDescent="0.2">
       <c r="A29" s="39"/>
       <c r="B29" s="6" t="s">
-        <v>54</v>
+        <v>52</v>
       </c>
       <c r="C29" s="7" t="s">
-        <v>13</v>
+        <v>15</v>
       </c>
       <c r="D29" s="7" t="s">
-        <v>20</v>
+        <v>6</v>
       </c>
       <c r="E29" s="10" t="s">
         <v>7</v>
@@ -4591,59 +4597,59 @@
       </c>
     </row>
     <row r="30" spans="1:8" ht="16" x14ac:dyDescent="0.2">
-      <c r="A30" s="39" t="s">
-        <v>56</v>
-      </c>
+      <c r="A30" s="39"/>
       <c r="B30" s="6" t="s">
-        <v>60</v>
+        <v>53</v>
       </c>
       <c r="C30" s="7" t="s">
-        <v>13</v>
+        <v>15</v>
       </c>
       <c r="D30" s="7" t="s">
-        <v>17</v>
+        <v>20</v>
       </c>
       <c r="E30" s="28" t="s">
         <v>22</v>
       </c>
       <c r="F30" s="28" t="s">
-        <v>83</v>
+        <v>85</v>
       </c>
       <c r="G30" s="5">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="H30" s="5" t="s">
-        <v>76</v>
+        <v>75</v>
       </c>
     </row>
     <row r="31" spans="1:8" ht="16" x14ac:dyDescent="0.2">
       <c r="A31" s="39"/>
       <c r="B31" s="6" t="s">
-        <v>61</v>
+        <v>54</v>
       </c>
       <c r="C31" s="7" t="s">
-        <v>10</v>
+        <v>13</v>
       </c>
       <c r="D31" s="7" t="s">
-        <v>17</v>
-      </c>
-      <c r="E31" s="28" t="s">
-        <v>22</v>
+        <v>20</v>
+      </c>
+      <c r="E31" s="10" t="s">
+        <v>7</v>
       </c>
       <c r="F31" s="28" t="s">
-        <v>83</v>
+        <v>85</v>
       </c>
       <c r="G31" s="5">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="H31" s="5" t="s">
-        <v>76</v>
+        <v>75</v>
       </c>
     </row>
     <row r="32" spans="1:8" ht="16" x14ac:dyDescent="0.2">
-      <c r="A32" s="39"/>
+      <c r="A32" s="39" t="s">
+        <v>56</v>
+      </c>
       <c r="B32" s="6" t="s">
-        <v>62</v>
+        <v>60</v>
       </c>
       <c r="C32" s="7" t="s">
         <v>13</v>
@@ -4664,60 +4670,60 @@
         <v>76</v>
       </c>
     </row>
-    <row r="33" spans="1:8" ht="16" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A33" s="39" t="s">
-        <v>57</v>
-      </c>
+    <row r="33" spans="1:8" ht="16" x14ac:dyDescent="0.2">
+      <c r="A33" s="39"/>
       <c r="B33" s="6" t="s">
-        <v>45</v>
+        <v>61</v>
       </c>
       <c r="C33" s="7" t="s">
-        <v>15</v>
+        <v>10</v>
       </c>
       <c r="D33" s="7" t="s">
-        <v>21</v>
-      </c>
-      <c r="E33" s="10" t="s">
+        <v>17</v>
+      </c>
+      <c r="E33" s="28" t="s">
         <v>22</v>
       </c>
       <c r="F33" s="28" t="s">
         <v>83</v>
       </c>
       <c r="G33" s="5">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="H33" s="5" t="s">
-        <v>75</v>
+        <v>76</v>
       </c>
     </row>
     <row r="34" spans="1:8" ht="16" x14ac:dyDescent="0.2">
       <c r="A34" s="39"/>
       <c r="B34" s="6" t="s">
-        <v>46</v>
+        <v>62</v>
       </c>
       <c r="C34" s="7" t="s">
-        <v>15</v>
+        <v>13</v>
       </c>
       <c r="D34" s="7" t="s">
-        <v>21</v>
-      </c>
-      <c r="E34" s="10" t="s">
+        <v>17</v>
+      </c>
+      <c r="E34" s="28" t="s">
         <v>22</v>
       </c>
       <c r="F34" s="28" t="s">
         <v>83</v>
       </c>
       <c r="G34" s="5">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="H34" s="5" t="s">
-        <v>75</v>
-      </c>
-    </row>
-    <row r="35" spans="1:8" ht="16" x14ac:dyDescent="0.2">
-      <c r="A35" s="39"/>
+        <v>76</v>
+      </c>
+    </row>
+    <row r="35" spans="1:8" ht="16" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A35" s="39" t="s">
+        <v>57</v>
+      </c>
       <c r="B35" s="6" t="s">
-        <v>47</v>
+        <v>45</v>
       </c>
       <c r="C35" s="7" t="s">
         <v>15</v>
@@ -4732,305 +4738,353 @@
         <v>83</v>
       </c>
       <c r="G35" s="5">
+        <v>2</v>
+      </c>
+      <c r="H35" s="5" t="s">
+        <v>75</v>
+      </c>
+    </row>
+    <row r="36" spans="1:8" ht="16" x14ac:dyDescent="0.2">
+      <c r="A36" s="39"/>
+      <c r="B36" s="6" t="s">
+        <v>46</v>
+      </c>
+      <c r="C36" s="7" t="s">
+        <v>15</v>
+      </c>
+      <c r="D36" s="7" t="s">
+        <v>21</v>
+      </c>
+      <c r="E36" s="10" t="s">
+        <v>22</v>
+      </c>
+      <c r="F36" s="28" t="s">
+        <v>83</v>
+      </c>
+      <c r="G36" s="5">
+        <v>2</v>
+      </c>
+      <c r="H36" s="5" t="s">
+        <v>75</v>
+      </c>
+    </row>
+    <row r="37" spans="1:8" ht="16" x14ac:dyDescent="0.2">
+      <c r="A37" s="39"/>
+      <c r="B37" s="6" t="s">
+        <v>47</v>
+      </c>
+      <c r="C37" s="7" t="s">
+        <v>15</v>
+      </c>
+      <c r="D37" s="7" t="s">
+        <v>21</v>
+      </c>
+      <c r="E37" s="10" t="s">
+        <v>22</v>
+      </c>
+      <c r="F37" s="28" t="s">
+        <v>83</v>
+      </c>
+      <c r="G37" s="5">
         <v>3</v>
       </c>
-      <c r="H35" s="5" t="s">
+      <c r="H37" s="5" t="s">
         <v>76</v>
       </c>
     </row>
-    <row r="36" spans="1:8" ht="16" x14ac:dyDescent="0.2">
-      <c r="A36" s="38" t="s">
+    <row r="38" spans="1:8" ht="16" x14ac:dyDescent="0.2">
+      <c r="A38" s="38" t="s">
         <v>65</v>
       </c>
-      <c r="B36" s="27" t="s">
+      <c r="B38" s="27" t="s">
         <v>63</v>
       </c>
-      <c r="C36" s="5" t="s">
+      <c r="C38" s="5" t="s">
         <v>16</v>
       </c>
-      <c r="D36" s="7" t="s">
+      <c r="D38" s="7" t="s">
         <v>6</v>
       </c>
-      <c r="E36" s="10" t="s">
+      <c r="E38" s="10" t="s">
         <v>7</v>
       </c>
-      <c r="F36" s="10" t="s">
+      <c r="F38" s="10" t="s">
         <v>86</v>
       </c>
-      <c r="G36" s="5">
+      <c r="G38" s="5">
         <v>1</v>
       </c>
-      <c r="H36" s="5" t="s">
+      <c r="H38" s="5" t="s">
         <v>74</v>
       </c>
     </row>
-    <row r="37" spans="1:8" ht="16" x14ac:dyDescent="0.2">
-      <c r="A37" s="38"/>
-      <c r="B37" s="27" t="s">
+    <row r="39" spans="1:8" ht="16" x14ac:dyDescent="0.2">
+      <c r="A39" s="38"/>
+      <c r="B39" s="27" t="s">
         <v>64</v>
       </c>
-      <c r="C37" s="5" t="s">
+      <c r="C39" s="5" t="s">
         <v>16</v>
       </c>
-      <c r="D37" s="7" t="s">
+      <c r="D39" s="7" t="s">
         <v>6</v>
       </c>
-      <c r="E37" s="10" t="s">
+      <c r="E39" s="10" t="s">
         <v>7</v>
       </c>
-      <c r="F37" s="10" t="s">
+      <c r="F39" s="10" t="s">
         <v>86</v>
       </c>
-      <c r="G37" s="5">
+      <c r="G39" s="5">
         <v>1</v>
       </c>
-      <c r="H37" s="5" t="s">
+      <c r="H39" s="5" t="s">
         <v>75</v>
       </c>
     </row>
-    <row r="38" spans="1:8" ht="16" x14ac:dyDescent="0.2">
-      <c r="B38" s="24" t="s">
+    <row r="40" spans="1:8" ht="16" x14ac:dyDescent="0.2">
+      <c r="B40" s="24" t="s">
         <v>2</v>
       </c>
-      <c r="C38" s="24" t="s">
+      <c r="C40" s="24" t="s">
         <v>5</v>
       </c>
-      <c r="D38" s="25" t="s">
+      <c r="D40" s="25" t="s">
         <v>23</v>
       </c>
-      <c r="E38" s="26" t="s">
+      <c r="E40" s="26" t="s">
         <v>24</v>
       </c>
-      <c r="F38" s="31"/>
-    </row>
-    <row r="39" spans="1:8" ht="16" x14ac:dyDescent="0.2">
-      <c r="B39" s="4" t="s">
+      <c r="F40" s="31"/>
+    </row>
+    <row r="41" spans="1:8" ht="16" x14ac:dyDescent="0.2">
+      <c r="B41" s="4" t="s">
         <v>8</v>
       </c>
-      <c r="C39" s="15" t="s">
+      <c r="C41" s="15" t="s">
         <v>9</v>
       </c>
-      <c r="D39" s="5">
-        <f>COUNTIF(C2:C37,"New Product Integration")</f>
+      <c r="D41" s="5">
+        <f>COUNTIF(C2:C39,"New Product Integration")</f>
         <v>1</v>
       </c>
-      <c r="E39" s="21">
-        <f t="shared" ref="E39:E44" si="0">D39/36</f>
+      <c r="E41" s="21">
+        <f t="shared" ref="E41:E46" si="0">D41/36</f>
         <v>2.7777777777777776E-2</v>
       </c>
-      <c r="F39" s="32"/>
-    </row>
-    <row r="40" spans="1:8" ht="16" x14ac:dyDescent="0.2">
-      <c r="B40" s="4" t="s">
+      <c r="F41" s="32"/>
+    </row>
+    <row r="42" spans="1:8" ht="16" x14ac:dyDescent="0.2">
+      <c r="B42" s="4" t="s">
         <v>10</v>
       </c>
-      <c r="C40" s="15" t="s">
+      <c r="C42" s="15" t="s">
         <v>9</v>
       </c>
-      <c r="D40" s="5">
-        <f>COUNTIF(C2:C37,"New Technical Integration")</f>
+      <c r="D42" s="5">
+        <f>COUNTIF(C2:C39,"New Technical Integration")</f>
         <v>2</v>
       </c>
-      <c r="E40" s="21">
+      <c r="E42" s="21">
         <f t="shared" si="0"/>
         <v>5.5555555555555552E-2</v>
       </c>
-      <c r="F40" s="32"/>
-    </row>
-    <row r="41" spans="1:8" ht="16" x14ac:dyDescent="0.2">
-      <c r="B41" s="4" t="s">
+      <c r="F42" s="32"/>
+    </row>
+    <row r="43" spans="1:8" ht="16" x14ac:dyDescent="0.2">
+      <c r="B43" s="4" t="s">
         <v>11</v>
       </c>
-      <c r="C41" s="14" t="s">
+      <c r="C43" s="14" t="s">
         <v>12</v>
       </c>
-      <c r="D41" s="5">
-        <f>COUNTIF(C2:C37,"New Interoperability Capability")</f>
+      <c r="D43" s="5">
+        <f>COUNTIF(C2:C39,"New Interoperability Capability")</f>
         <v>0</v>
       </c>
-      <c r="E41" s="21">
+      <c r="E43" s="21">
         <f t="shared" si="0"/>
         <v>0</v>
       </c>
-      <c r="F41" s="32"/>
-    </row>
-    <row r="42" spans="1:8" ht="16" x14ac:dyDescent="0.2">
-      <c r="B42" s="4" t="s">
-        <v>13</v>
-      </c>
-      <c r="C42" s="16" t="s">
-        <v>14</v>
-      </c>
-      <c r="D42" s="5">
-        <f>COUNTIF(C2:C37,"New Feature Introduction")</f>
-        <v>23</v>
-      </c>
-      <c r="E42" s="21">
-        <f t="shared" si="0"/>
-        <v>0.63888888888888884</v>
-      </c>
-      <c r="F42" s="32"/>
-    </row>
-    <row r="43" spans="1:8" ht="16" x14ac:dyDescent="0.2">
-      <c r="B43" s="4" t="s">
-        <v>15</v>
-      </c>
-      <c r="C43" s="16" t="s">
-        <v>14</v>
-      </c>
-      <c r="D43" s="5">
-        <f>COUNTIF(C2:C37,"New Function Introduction")</f>
-        <v>8</v>
-      </c>
-      <c r="E43" s="21">
-        <f t="shared" si="0"/>
-        <v>0.22222222222222221</v>
-      </c>
       <c r="F43" s="32"/>
     </row>
     <row r="44" spans="1:8" ht="16" x14ac:dyDescent="0.2">
       <c r="B44" s="4" t="s">
-        <v>16</v>
-      </c>
-      <c r="C44" s="14" t="s">
-        <v>12</v>
+        <v>13</v>
+      </c>
+      <c r="C44" s="16" t="s">
+        <v>14</v>
       </c>
       <c r="D44" s="5">
-        <f>COUNTIF(C2:C37,"Sustaining")</f>
-        <v>2</v>
+        <f>COUNTIF(C2:C39,"New Feature Introduction")</f>
+        <v>24</v>
       </c>
       <c r="E44" s="21">
         <f t="shared" si="0"/>
+        <v>0.66666666666666663</v>
+      </c>
+      <c r="F44" s="32"/>
+    </row>
+    <row r="45" spans="1:8" ht="16" x14ac:dyDescent="0.2">
+      <c r="B45" s="4" t="s">
+        <v>15</v>
+      </c>
+      <c r="C45" s="16" t="s">
+        <v>14</v>
+      </c>
+      <c r="D45" s="5">
+        <f>COUNTIF(C2:C39,"New Function Introduction")</f>
+        <v>9</v>
+      </c>
+      <c r="E45" s="21">
+        <f t="shared" si="0"/>
+        <v>0.25</v>
+      </c>
+      <c r="F45" s="32"/>
+    </row>
+    <row r="46" spans="1:8" ht="16" x14ac:dyDescent="0.2">
+      <c r="B46" s="4" t="s">
+        <v>16</v>
+      </c>
+      <c r="C46" s="14" t="s">
+        <v>12</v>
+      </c>
+      <c r="D46" s="5">
+        <f>COUNTIF(C2:C39,"Sustaining")</f>
+        <v>2</v>
+      </c>
+      <c r="E46" s="21">
+        <f t="shared" si="0"/>
         <v>5.5555555555555552E-2</v>
       </c>
-      <c r="F44" s="32"/>
-    </row>
-    <row r="46" spans="1:8" ht="16" x14ac:dyDescent="0.2">
-      <c r="B46" s="3" t="s">
+      <c r="F46" s="32"/>
+    </row>
+    <row r="48" spans="1:8" ht="16" x14ac:dyDescent="0.2">
+      <c r="B48" s="3" t="s">
         <v>18</v>
       </c>
-      <c r="C46" s="17" t="s">
+      <c r="C48" s="17" t="s">
         <v>23</v>
       </c>
-      <c r="D46" s="13" t="s">
+      <c r="D48" s="13" t="s">
         <v>24</v>
-      </c>
-    </row>
-    <row r="47" spans="1:8" x14ac:dyDescent="0.2">
-      <c r="B47" s="14" t="s">
-        <v>19</v>
-      </c>
-      <c r="C47" s="14">
-        <f>COUNTIF(D2:D37,"Energy &amp; Sustainability")</f>
-        <v>4</v>
-      </c>
-      <c r="D47" s="20">
-        <f>C47/36</f>
-        <v>0.1111111111111111</v>
-      </c>
-    </row>
-    <row r="48" spans="1:8" x14ac:dyDescent="0.2">
-      <c r="B48" s="14" t="s">
-        <v>20</v>
-      </c>
-      <c r="C48" s="14">
-        <f>COUNTIF(D2:D37,"Ease of Use &amp; Accessibility")</f>
-        <v>7</v>
-      </c>
-      <c r="D48" s="20">
-        <f>C48/36</f>
-        <v>0.19444444444444445</v>
       </c>
     </row>
     <row r="49" spans="1:4" x14ac:dyDescent="0.2">
       <c r="B49" s="14" t="s">
-        <v>6</v>
+        <v>19</v>
       </c>
       <c r="C49" s="14">
-        <f>COUNTIF(D2:D37,"Trust, Security &amp; Reliability")</f>
-        <v>11</v>
+        <f>COUNTIF(D2:D39,"Energy &amp; Sustainability")</f>
+        <v>4</v>
       </c>
       <c r="D49" s="20">
         <f>C49/36</f>
-        <v>0.30555555555555558</v>
+        <v>0.1111111111111111</v>
       </c>
     </row>
     <row r="50" spans="1:4" x14ac:dyDescent="0.2">
       <c r="B50" s="14" t="s">
-        <v>17</v>
+        <v>20</v>
       </c>
       <c r="C50" s="14">
-        <f>COUNTIF(D2:D37,"Intelligence &amp; Automation")</f>
-        <v>8</v>
+        <f>COUNTIF(D2:D39,"Ease of Use &amp; Accessibility")</f>
+        <v>7</v>
       </c>
       <c r="D50" s="20">
         <f>C50/36</f>
-        <v>0.22222222222222221</v>
+        <v>0.19444444444444445</v>
       </c>
     </row>
     <row r="51" spans="1:4" x14ac:dyDescent="0.2">
       <c r="B51" s="14" t="s">
-        <v>21</v>
+        <v>6</v>
       </c>
       <c r="C51" s="14">
-        <f>COUNTIF(D2:D37,"Engagement &amp; Personalization")</f>
-        <v>6</v>
+        <f>COUNTIF(D2:D39,"Trust, Security &amp; Reliability")</f>
+        <v>12</v>
       </c>
       <c r="D51" s="20">
         <f>C51/36</f>
+        <v>0.33333333333333331</v>
+      </c>
+    </row>
+    <row r="52" spans="1:4" x14ac:dyDescent="0.2">
+      <c r="B52" s="14" t="s">
+        <v>17</v>
+      </c>
+      <c r="C52" s="14">
+        <f>COUNTIF(D2:D39,"Intelligence &amp; Automation")</f>
+        <v>9</v>
+      </c>
+      <c r="D52" s="20">
+        <f>C52/36</f>
+        <v>0.25</v>
+      </c>
+    </row>
+    <row r="53" spans="1:4" x14ac:dyDescent="0.2">
+      <c r="B53" s="14" t="s">
+        <v>21</v>
+      </c>
+      <c r="C53" s="14">
+        <f>COUNTIF(D2:D39,"Engagement &amp; Personalization")</f>
+        <v>6</v>
+      </c>
+      <c r="D53" s="20">
+        <f>C53/36</f>
         <v>0.16666666666666666</v>
       </c>
     </row>
-    <row r="53" spans="1:4" ht="16" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="B53" s="12" t="s">
+    <row r="55" spans="1:4" ht="16" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="B55" s="12" t="s">
         <v>4</v>
       </c>
-      <c r="C53" s="18" t="s">
+      <c r="C55" s="18" t="s">
         <v>23</v>
       </c>
-      <c r="D53" s="13" t="s">
+      <c r="D55" s="13" t="s">
         <v>24</v>
       </c>
     </row>
-    <row r="54" spans="1:4" s="11" customFormat="1" x14ac:dyDescent="0.2">
-      <c r="A54" s="1"/>
-      <c r="B54" s="10" t="s">
+    <row r="56" spans="1:4" s="11" customFormat="1" x14ac:dyDescent="0.2">
+      <c r="A56" s="1"/>
+      <c r="B56" s="10" t="s">
         <v>7</v>
       </c>
-      <c r="C54" s="19">
-        <f>COUNTIF(E2:E37,"Basic (Free)")</f>
-        <v>25</v>
-      </c>
-      <c r="D54" s="20">
-        <f>C54/36</f>
-        <v>0.69444444444444442</v>
-      </c>
-    </row>
-    <row r="55" spans="1:4" s="11" customFormat="1" x14ac:dyDescent="0.2">
-      <c r="A55" s="1"/>
-      <c r="B55" s="10" t="s">
+      <c r="C56" s="19">
+        <f>COUNTIF(E2:E39,"Basic (Free)")</f>
+        <v>26</v>
+      </c>
+      <c r="D56" s="20">
+        <f>C56/36</f>
+        <v>0.72222222222222221</v>
+      </c>
+    </row>
+    <row r="57" spans="1:4" s="11" customFormat="1" x14ac:dyDescent="0.2">
+      <c r="A57" s="1"/>
+      <c r="B57" s="10" t="s">
         <v>22</v>
       </c>
-      <c r="C55" s="14">
-        <f>COUNTIF(E2:E37,"Paid")</f>
-        <v>11</v>
-      </c>
-      <c r="D55" s="20">
-        <f>C55/36</f>
-        <v>0.30555555555555558</v>
+      <c r="C57" s="14">
+        <f>COUNTIF(E2:E39,"Paid")</f>
+        <v>12</v>
+      </c>
+      <c r="D57" s="20">
+        <f>C57/36</f>
+        <v>0.33333333333333331</v>
       </c>
     </row>
   </sheetData>
   <mergeCells count="9">
-    <mergeCell ref="A14:A17"/>
+    <mergeCell ref="A15:A18"/>
     <mergeCell ref="A2:A9"/>
-    <mergeCell ref="A36:A37"/>
-    <mergeCell ref="A30:A32"/>
-    <mergeCell ref="A33:A35"/>
-    <mergeCell ref="A10:A13"/>
-    <mergeCell ref="A18:A21"/>
-    <mergeCell ref="A26:A29"/>
-    <mergeCell ref="A22:A25"/>
+    <mergeCell ref="A38:A39"/>
+    <mergeCell ref="A32:A34"/>
+    <mergeCell ref="A35:A37"/>
+    <mergeCell ref="A10:A14"/>
+    <mergeCell ref="A19:A23"/>
+    <mergeCell ref="A28:A31"/>
+    <mergeCell ref="A24:A27"/>
   </mergeCells>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>